<commit_message>
feat: Implement category API and redesign authentication and cake listing pages with new category tabs and enhanced cake cards.
</commit_message>
<xml_diff>
--- a/doanmon/FILE_1_MAU_IMPORT_BANH.xlsx
+++ b/doanmon/FILE_1_MAU_IMPORT_BANH.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="46" uniqueCount="39">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="46" uniqueCount="40">
   <si>
     <t>productCode</t>
   </si>
@@ -32,103 +32,106 @@
     <t>description</t>
   </si>
   <si>
-    <t>CAKE-CHOCO-001</t>
-  </si>
-  <si>
-    <t>Chocolate Fudge Cake</t>
-  </si>
-  <si>
-    <t>Chocolate</t>
-  </si>
-  <si>
-    <t>Rich dark chocolate cake with fudge frosting</t>
-  </si>
-  <si>
-    <t>CAKE-CHOCO-002</t>
-  </si>
-  <si>
-    <t>Chocolate Truffle Delight</t>
-  </si>
-  <si>
-    <t>Premium chocolate truffle cake</t>
-  </si>
-  <si>
-    <t>CAKE-CHOCO-003</t>
-  </si>
-  <si>
-    <t>Double Chocolate Dream</t>
-  </si>
-  <si>
-    <t>Double layer chocolate sponge</t>
-  </si>
-  <si>
-    <t>CAKE-VANILLA-001</t>
-  </si>
-  <si>
-    <t>Classic Vanilla Sponge</t>
-  </si>
-  <si>
-    <t>Vanilla</t>
-  </si>
-  <si>
-    <t>Light and fluffy vanilla cake</t>
-  </si>
-  <si>
-    <t>CAKE-VANILLA-002</t>
-  </si>
-  <si>
-    <t>Vanilla Bean Supreme</t>
-  </si>
-  <si>
-    <t>Made with real vanilla beans</t>
-  </si>
-  <si>
-    <t>CAKE-FRUIT-001</t>
-  </si>
-  <si>
-    <t>Strawberry Shortcake</t>
-  </si>
-  <si>
-    <t>Fruit</t>
-  </si>
-  <si>
-    <t>Fresh strawberries with cream</t>
-  </si>
-  <si>
-    <t>CAKE-FRUIT-002</t>
-  </si>
-  <si>
-    <t>Blueberry Bliss</t>
-  </si>
-  <si>
-    <t>Loaded with fresh blueberries</t>
-  </si>
-  <si>
-    <t>CAKE-FRUIT-003</t>
-  </si>
-  <si>
-    <t>Mixed Berry Delight</t>
-  </si>
-  <si>
-    <t>Strawberry raspberry and blueberry mix</t>
-  </si>
-  <si>
-    <t>CAKE-SPECIAL-001</t>
-  </si>
-  <si>
-    <t>Red Velvet Classic</t>
-  </si>
-  <si>
-    <t>Traditional red velvet with cream cheese</t>
-  </si>
-  <si>
-    <t>CAKE-SPECIAL-002</t>
-  </si>
-  <si>
-    <t>Carrot Cake Supreme</t>
-  </si>
-  <si>
-    <t>Moist carrot cake with walnuts</t>
+    <t>CAKE-BDAY-001</t>
+  </si>
+  <si>
+    <t>Rainbow Birthday Cake</t>
+  </si>
+  <si>
+    <t>Birthday Cakes</t>
+  </si>
+  <si>
+    <t>Colorful rainbow layers perfect for birthdays</t>
+  </si>
+  <si>
+    <t>CAKE-BDAY-002</t>
+  </si>
+  <si>
+    <t>Unicorn Dream Cake</t>
+  </si>
+  <si>
+    <t>Magical unicorn themed birthday cake</t>
+  </si>
+  <si>
+    <t>CAKE-BDAY-003</t>
+  </si>
+  <si>
+    <t>Chocolate Birthday Delight</t>
+  </si>
+  <si>
+    <t>Rich chocolate birthday cake with sprinkles</t>
+  </si>
+  <si>
+    <t>CAKE-WEDDING-001</t>
+  </si>
+  <si>
+    <t>Classic White Wedding Cake</t>
+  </si>
+  <si>
+    <t>Wedding Cakes</t>
+  </si>
+  <si>
+    <t>Elegant 3-tier white wedding cake</t>
+  </si>
+  <si>
+    <t>CAKE-WEDDING-002</t>
+  </si>
+  <si>
+    <t>Rose Garden Wedding Cake</t>
+  </si>
+  <si>
+    <t>Beautiful rose decorated wedding cake</t>
+  </si>
+  <si>
+    <t>CAKE-CHEESE-001</t>
+  </si>
+  <si>
+    <t>New York Cheesecake</t>
+  </si>
+  <si>
+    <t>Cheese Cakes</t>
+  </si>
+  <si>
+    <t>Classic creamy New York style cheesecake</t>
+  </si>
+  <si>
+    <t>CAKE-CHEESE-002</t>
+  </si>
+  <si>
+    <t>Blueberry Cheesecake</t>
+  </si>
+  <si>
+    <t>Cheesecake with fresh blueberry topping</t>
+  </si>
+  <si>
+    <t>CAKE-CHEESE-003</t>
+  </si>
+  <si>
+    <t>Strawberry Cheesecake</t>
+  </si>
+  <si>
+    <t>Cheesecake with strawberry compote</t>
+  </si>
+  <si>
+    <t>CAKE-GATAUX-001</t>
+  </si>
+  <si>
+    <t>Black Forest Gataux</t>
+  </si>
+  <si>
+    <t>Gataux</t>
+  </si>
+  <si>
+    <t>Traditional Black Forest gataux with cherries</t>
+  </si>
+  <si>
+    <t>CAKE-GATAUX-002</t>
+  </si>
+  <si>
+    <t>Opera Gataux</t>
+  </si>
+  <si>
+    <t>French opera gataux with coffee and chocolate</t>
   </si>
 </sst>
 </file>
@@ -192,12 +195,12 @@
   <dimension ref="A1:F11"/>
   <sheetFormatPr defaultRowHeight="15.0"/>
   <cols>
-    <col min="1" max="1" width="16.33203125" customWidth="true" bestFit="true"/>
-    <col min="2" max="2" width="20.203125" customWidth="true" bestFit="true"/>
+    <col min="1" max="1" width="17.15234375" customWidth="true" bestFit="true"/>
+    <col min="2" max="2" width="22.390625" customWidth="true" bestFit="true"/>
     <col min="3" max="3" width="5.46875" customWidth="true" bestFit="true"/>
     <col min="4" max="4" width="13.75" customWidth="true" bestFit="true"/>
     <col min="5" max="5" width="8.44140625" customWidth="true" bestFit="true"/>
-    <col min="6" max="6" width="35.125" customWidth="true" bestFit="true"/>
+    <col min="6" max="6" width="36.84765625" customWidth="true" bestFit="true"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -228,7 +231,7 @@
         <v>7</v>
       </c>
       <c r="C2" t="n" s="0">
-        <v>28.99</v>
+        <v>35.99</v>
       </c>
       <c r="D2" t="s" s="0">
         <v>8</v>
@@ -248,7 +251,7 @@
         <v>11</v>
       </c>
       <c r="C3" t="n" s="0">
-        <v>32.5</v>
+        <v>42.5</v>
       </c>
       <c r="D3" t="s" s="0">
         <v>8</v>
@@ -268,7 +271,7 @@
         <v>14</v>
       </c>
       <c r="C4" t="n" s="0">
-        <v>26.75</v>
+        <v>38.75</v>
       </c>
       <c r="D4" t="s" s="0">
         <v>8</v>
@@ -288,13 +291,13 @@
         <v>17</v>
       </c>
       <c r="C5" t="n" s="0">
-        <v>18.99</v>
+        <v>150.0</v>
       </c>
       <c r="D5" t="s" s="0">
         <v>18</v>
       </c>
       <c r="E5" t="n" s="0">
-        <v>60.0</v>
+        <v>15.0</v>
       </c>
       <c r="F5" t="s" s="0">
         <v>19</v>
@@ -308,13 +311,13 @@
         <v>21</v>
       </c>
       <c r="C6" t="n" s="0">
-        <v>22.5</v>
+        <v>180.0</v>
       </c>
       <c r="D6" t="s" s="0">
         <v>18</v>
       </c>
       <c r="E6" t="n" s="0">
-        <v>35.0</v>
+        <v>10.0</v>
       </c>
       <c r="F6" t="s" s="0">
         <v>22</v>
@@ -328,7 +331,7 @@
         <v>24</v>
       </c>
       <c r="C7" t="n" s="0">
-        <v>24.99</v>
+        <v>28.99</v>
       </c>
       <c r="D7" t="s" s="0">
         <v>25</v>
@@ -348,7 +351,7 @@
         <v>28</v>
       </c>
       <c r="C8" t="n" s="0">
-        <v>23.5</v>
+        <v>32.5</v>
       </c>
       <c r="D8" t="s" s="0">
         <v>25</v>
@@ -368,13 +371,13 @@
         <v>31</v>
       </c>
       <c r="C9" t="n" s="0">
-        <v>25.99</v>
+        <v>32.5</v>
       </c>
       <c r="D9" t="s" s="0">
         <v>25</v>
       </c>
       <c r="E9" t="n" s="0">
-        <v>30.0</v>
+        <v>35.0</v>
       </c>
       <c r="F9" t="s" s="0">
         <v>32</v>
@@ -388,36 +391,36 @@
         <v>34</v>
       </c>
       <c r="C10" t="n" s="0">
-        <v>29.99</v>
+        <v>45.99</v>
       </c>
       <c r="D10" t="s" s="0">
-        <v>8</v>
+        <v>35</v>
       </c>
       <c r="E10" t="n" s="0">
         <v>25.0</v>
       </c>
       <c r="F10" t="s" s="0">
-        <v>35</v>
+        <v>36</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="s" s="0">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="B11" t="s" s="0">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="C11" t="n" s="0">
-        <v>27.5</v>
+        <v>48.5</v>
       </c>
       <c r="D11" t="s" s="0">
-        <v>18</v>
+        <v>35</v>
       </c>
       <c r="E11" t="n" s="0">
         <v>20.0</v>
       </c>
       <c r="F11" t="s" s="0">
-        <v>38</v>
+        <v>39</v>
       </c>
     </row>
   </sheetData>

</xml_diff>